<commit_message>
Added new content from recent stream.
</commit_message>
<xml_diff>
--- a/_Projects/P1012202501-ESP32_Stepper_Controller/ProjectDocuments/test-logs/P1012202501-01 Test Plan Log.xlsx
+++ b/_Projects/P1012202501-ESP32_Stepper_Controller/ProjectDocuments/test-logs/P1012202501-01 Test Plan Log.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="99">
   <si>
     <t xml:space="preserve">Initial Testing</t>
   </si>
@@ -172,7 +172,151 @@
     <t xml:space="preserve">Test 24</t>
   </si>
   <si>
+    <t xml:space="preserve">Is the resistance between CN4 Terminal 1 and Terminal 4 &gt;= 1KΩ?</t>
+  </si>
+  <si>
     <t xml:space="preserve">Test 25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between CN4 Terminal 2 and Terminal 4 &gt;= 1KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between CN4 Terminal 3 and Terminal 4 &gt;= 1KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between CN4 Terminal 1 and Terminal 2 &gt;= 1KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between CN4 Terminal 1 and Terminal 3 &gt;= 1KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between CN4 Terminal 2 and Terminal 3 &gt;= 1KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between TP24 and TP25 &gt;= 5KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between TP22 and TP23 &gt;= 1KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between TP18 and TP19 &gt;= 1KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between TP20 and TP21 &gt;= 1KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between CN7 Terminal 1 and TP7 &gt;= 5KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between CN7 Terminal 2 and TP7 &gt;= 5KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between CN7 Terminal 3 and TP7 &gt;= 5KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between CN7 Terminal 4 and TP7 &gt;= 5KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between CN7 Terminal 1 and Terminal 4 &gt;= 5KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between CN7 Terminal 2 and Terminal 4 &gt;= 5KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between CN7 Terminal 3 and Terminal 4 &gt;= 5KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between CN7 Terminal 1 and Terminal 3 &gt;= 5KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between CN7 Terminal 2 and Terminal 3 &gt;= 5KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the resistance between CN7 Terminal 1 and Terminal 2 &gt;= 5KΩ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the PCB assembly pass the low voltage and limited current test?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the PCB assembly pass the operational voltage test?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the 3.3V power supply output the proper voltage within tolerance?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the 5.0V power supply output the proper voltage within tolerance?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 49</t>
   </si>
 </sst>
 </file>
@@ -473,7 +617,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A6:R43"/>
+  <dimension ref="A6:R57"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -579,15 +723,15 @@
         <v>9</v>
       </c>
       <c r="B10" s="3"/>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
@@ -603,15 +747,15 @@
         <v>11</v>
       </c>
       <c r="B11" s="3"/>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
       <c r="J11" s="4"/>
       <c r="K11" s="4"/>
       <c r="L11" s="4"/>
@@ -627,15 +771,15 @@
         <v>13</v>
       </c>
       <c r="B12" s="3"/>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
       <c r="J12" s="4"/>
       <c r="K12" s="4"/>
       <c r="L12" s="4"/>
@@ -651,15 +795,15 @@
         <v>15</v>
       </c>
       <c r="B13" s="3"/>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
       <c r="L13" s="4"/>
@@ -675,15 +819,15 @@
         <v>17</v>
       </c>
       <c r="B14" s="3"/>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
       <c r="L14" s="4"/>
@@ -699,15 +843,15 @@
         <v>19</v>
       </c>
       <c r="B15" s="3"/>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
       <c r="L15" s="4"/>
@@ -723,15 +867,15 @@
         <v>21</v>
       </c>
       <c r="B16" s="3"/>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
       <c r="L16" s="4"/>
@@ -747,15 +891,15 @@
         <v>23</v>
       </c>
       <c r="B17" s="3"/>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
       <c r="L17" s="4"/>
@@ -771,15 +915,15 @@
         <v>25</v>
       </c>
       <c r="B18" s="3"/>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
       <c r="J18" s="4"/>
       <c r="K18" s="4"/>
       <c r="L18" s="4"/>
@@ -795,15 +939,15 @@
         <v>27</v>
       </c>
       <c r="B19" s="3"/>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
       <c r="J19" s="4"/>
       <c r="K19" s="4"/>
       <c r="L19" s="4"/>
@@ -819,15 +963,15 @@
         <v>29</v>
       </c>
       <c r="B20" s="3"/>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
       <c r="L20" s="4"/>
@@ -843,15 +987,15 @@
         <v>31</v>
       </c>
       <c r="B21" s="3"/>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
       <c r="J21" s="4"/>
       <c r="K21" s="4"/>
       <c r="L21" s="4"/>
@@ -867,15 +1011,15 @@
         <v>33</v>
       </c>
       <c r="B22" s="3"/>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
       <c r="J22" s="4"/>
       <c r="K22" s="4"/>
       <c r="L22" s="4"/>
@@ -891,15 +1035,15 @@
         <v>35</v>
       </c>
       <c r="B23" s="3"/>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
       <c r="J23" s="4"/>
       <c r="K23" s="4"/>
       <c r="L23" s="4"/>
@@ -915,15 +1059,15 @@
         <v>36</v>
       </c>
       <c r="B24" s="3"/>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
       <c r="J24" s="4"/>
       <c r="K24" s="4"/>
       <c r="L24" s="4"/>
@@ -939,15 +1083,15 @@
         <v>37</v>
       </c>
       <c r="B25" s="3"/>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="5"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
       <c r="J25" s="4"/>
       <c r="K25" s="4"/>
       <c r="L25" s="4"/>
@@ -963,15 +1107,15 @@
         <v>39</v>
       </c>
       <c r="B26" s="3"/>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="5"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
       <c r="J26" s="4"/>
       <c r="K26" s="4"/>
       <c r="L26" s="4"/>
@@ -987,15 +1131,15 @@
         <v>41</v>
       </c>
       <c r="B27" s="3"/>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="5"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
       <c r="J27" s="4"/>
       <c r="K27" s="4"/>
       <c r="L27" s="4"/>
@@ -1011,15 +1155,15 @@
         <v>43</v>
       </c>
       <c r="B28" s="3"/>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5"/>
-      <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
       <c r="J28" s="4"/>
       <c r="K28" s="4"/>
       <c r="L28" s="4"/>
@@ -1035,15 +1179,15 @@
         <v>45</v>
       </c>
       <c r="B29" s="3"/>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="5"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
       <c r="J29" s="4"/>
       <c r="K29" s="4"/>
       <c r="L29" s="4"/>
@@ -1059,15 +1203,15 @@
         <v>47</v>
       </c>
       <c r="B30" s="3"/>
-      <c r="C30" s="5" t="s">
+      <c r="C30" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="5"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
       <c r="J30" s="4"/>
       <c r="K30" s="4"/>
       <c r="L30" s="4"/>
@@ -1083,7 +1227,9 @@
         <v>49</v>
       </c>
       <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
+      <c r="C31" s="3" t="s">
+        <v>50</v>
+      </c>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
@@ -1102,16 +1248,18 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
-      <c r="I32" s="3"/>
+      <c r="C32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+      <c r="I32" s="5"/>
       <c r="J32" s="4"/>
       <c r="K32" s="4"/>
       <c r="L32" s="4"/>
@@ -1123,15 +1271,19 @@
       <c r="R32" s="4"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3"/>
+      <c r="A33" s="3" t="s">
+        <v>53</v>
+      </c>
       <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
-      <c r="I33" s="3"/>
+      <c r="C33" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
       <c r="J33" s="4"/>
       <c r="K33" s="4"/>
       <c r="L33" s="4"/>
@@ -1143,15 +1295,19 @@
       <c r="R33" s="4"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3"/>
+      <c r="A34" s="3" t="s">
+        <v>55</v>
+      </c>
       <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
-      <c r="E34" s="3"/>
-      <c r="F34" s="3"/>
-      <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
-      <c r="I34" s="3"/>
+      <c r="C34" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="5"/>
+      <c r="I34" s="5"/>
       <c r="J34" s="4"/>
       <c r="K34" s="4"/>
       <c r="L34" s="4"/>
@@ -1163,15 +1319,19 @@
       <c r="R34" s="4"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3"/>
+      <c r="A35" s="3" t="s">
+        <v>57</v>
+      </c>
       <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
-      <c r="F35" s="3"/>
-      <c r="G35" s="3"/>
-      <c r="H35" s="3"/>
-      <c r="I35" s="3"/>
+      <c r="C35" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+      <c r="I35" s="5"/>
       <c r="J35" s="4"/>
       <c r="K35" s="4"/>
       <c r="L35" s="4"/>
@@ -1183,15 +1343,19 @@
       <c r="R35" s="4"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3"/>
+      <c r="A36" s="3" t="s">
+        <v>59</v>
+      </c>
       <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
-      <c r="F36" s="3"/>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
-      <c r="I36" s="3"/>
+      <c r="C36" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5"/>
+      <c r="I36" s="5"/>
       <c r="J36" s="4"/>
       <c r="K36" s="4"/>
       <c r="L36" s="4"/>
@@ -1203,9 +1367,13 @@
       <c r="R36" s="4"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="3"/>
+      <c r="A37" s="3" t="s">
+        <v>61</v>
+      </c>
       <c r="B37" s="3"/>
-      <c r="C37" s="3"/>
+      <c r="C37" s="3" t="s">
+        <v>62</v>
+      </c>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
@@ -1223,9 +1391,13 @@
       <c r="R37" s="4"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="3"/>
+      <c r="A38" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="B38" s="3"/>
-      <c r="C38" s="3"/>
+      <c r="C38" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
@@ -1243,9 +1415,13 @@
       <c r="R38" s="4"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3"/>
+      <c r="A39" s="3" t="s">
+        <v>65</v>
+      </c>
       <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
+      <c r="C39" s="3" t="s">
+        <v>66</v>
+      </c>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
@@ -1263,9 +1439,13 @@
       <c r="R39" s="4"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3"/>
+      <c r="A40" s="3" t="s">
+        <v>67</v>
+      </c>
       <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
+      <c r="C40" s="3" t="s">
+        <v>68</v>
+      </c>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
@@ -1283,9 +1463,13 @@
       <c r="R40" s="4"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="3"/>
+      <c r="A41" s="3" t="s">
+        <v>69</v>
+      </c>
       <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
+      <c r="C41" s="3" t="s">
+        <v>70</v>
+      </c>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
@@ -1303,9 +1487,13 @@
       <c r="R41" s="4"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3"/>
+      <c r="A42" s="3" t="s">
+        <v>71</v>
+      </c>
       <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
+      <c r="C42" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
@@ -1323,9 +1511,13 @@
       <c r="R42" s="4"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3"/>
+      <c r="A43" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="B43" s="3"/>
-      <c r="C43" s="3"/>
+      <c r="C43" s="3" t="s">
+        <v>74</v>
+      </c>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
@@ -1342,8 +1534,336 @@
       <c r="Q43" s="4"/>
       <c r="R43" s="4"/>
     </row>
+    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B44" s="3"/>
+      <c r="C44" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+      <c r="I44" s="3"/>
+      <c r="J44" s="4"/>
+      <c r="K44" s="4"/>
+      <c r="L44" s="4"/>
+      <c r="M44" s="4"/>
+      <c r="N44" s="4"/>
+      <c r="O44" s="4"/>
+      <c r="P44" s="4"/>
+      <c r="Q44" s="4"/>
+      <c r="R44" s="4"/>
+    </row>
+    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B45" s="3"/>
+      <c r="C45" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="4"/>
+      <c r="K45" s="4"/>
+      <c r="L45" s="4"/>
+      <c r="M45" s="4"/>
+      <c r="N45" s="4"/>
+      <c r="O45" s="4"/>
+      <c r="P45" s="4"/>
+      <c r="Q45" s="4"/>
+      <c r="R45" s="4"/>
+    </row>
+    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B46" s="3"/>
+      <c r="C46" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+      <c r="I46" s="3"/>
+      <c r="J46" s="4"/>
+      <c r="K46" s="4"/>
+      <c r="L46" s="4"/>
+      <c r="M46" s="4"/>
+      <c r="N46" s="4"/>
+      <c r="O46" s="4"/>
+      <c r="P46" s="4"/>
+      <c r="Q46" s="4"/>
+      <c r="R46" s="4"/>
+    </row>
+    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B47" s="3"/>
+      <c r="C47" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="4"/>
+      <c r="K47" s="4"/>
+      <c r="L47" s="4"/>
+      <c r="M47" s="4"/>
+      <c r="N47" s="4"/>
+      <c r="O47" s="4"/>
+      <c r="P47" s="4"/>
+      <c r="Q47" s="4"/>
+      <c r="R47" s="4"/>
+    </row>
+    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B48" s="3"/>
+      <c r="C48" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+      <c r="I48" s="3"/>
+      <c r="J48" s="4"/>
+      <c r="K48" s="4"/>
+      <c r="L48" s="4"/>
+      <c r="M48" s="4"/>
+      <c r="N48" s="4"/>
+      <c r="O48" s="4"/>
+      <c r="P48" s="4"/>
+      <c r="Q48" s="4"/>
+      <c r="R48" s="4"/>
+    </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B49" s="3"/>
+      <c r="C49" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+      <c r="I49" s="3"/>
+      <c r="J49" s="4"/>
+      <c r="K49" s="4"/>
+      <c r="L49" s="4"/>
+      <c r="M49" s="4"/>
+      <c r="N49" s="4"/>
+      <c r="O49" s="4"/>
+      <c r="P49" s="4"/>
+      <c r="Q49" s="4"/>
+      <c r="R49" s="4"/>
+    </row>
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B50" s="3"/>
+      <c r="C50" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
+      <c r="I50" s="3"/>
+      <c r="J50" s="4"/>
+      <c r="K50" s="4"/>
+      <c r="L50" s="4"/>
+      <c r="M50" s="4"/>
+      <c r="N50" s="4"/>
+      <c r="O50" s="4"/>
+      <c r="P50" s="4"/>
+      <c r="Q50" s="4"/>
+      <c r="R50" s="4"/>
+    </row>
+    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B51" s="3"/>
+      <c r="C51" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="3"/>
+      <c r="J51" s="4"/>
+      <c r="K51" s="4"/>
+      <c r="L51" s="4"/>
+      <c r="M51" s="4"/>
+      <c r="N51" s="4"/>
+      <c r="O51" s="4"/>
+      <c r="P51" s="4"/>
+      <c r="Q51" s="4"/>
+      <c r="R51" s="4"/>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B52" s="3"/>
+      <c r="C52" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="3"/>
+      <c r="I52" s="3"/>
+      <c r="J52" s="4"/>
+      <c r="K52" s="4"/>
+      <c r="L52" s="4"/>
+      <c r="M52" s="4"/>
+      <c r="N52" s="4"/>
+      <c r="O52" s="4"/>
+      <c r="P52" s="4"/>
+      <c r="Q52" s="4"/>
+      <c r="R52" s="4"/>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B53" s="3"/>
+      <c r="C53" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="D53" s="3"/>
+      <c r="E53" s="3"/>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3"/>
+      <c r="H53" s="3"/>
+      <c r="I53" s="3"/>
+      <c r="J53" s="4"/>
+      <c r="K53" s="4"/>
+      <c r="L53" s="4"/>
+      <c r="M53" s="4"/>
+      <c r="N53" s="4"/>
+      <c r="O53" s="4"/>
+      <c r="P53" s="4"/>
+      <c r="Q53" s="4"/>
+      <c r="R53" s="4"/>
+    </row>
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B54" s="3"/>
+      <c r="C54" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D54" s="3"/>
+      <c r="E54" s="3"/>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="3"/>
+      <c r="I54" s="3"/>
+      <c r="J54" s="4"/>
+      <c r="K54" s="4"/>
+      <c r="L54" s="4"/>
+      <c r="M54" s="4"/>
+      <c r="N54" s="4"/>
+      <c r="O54" s="4"/>
+      <c r="P54" s="4"/>
+      <c r="Q54" s="4"/>
+      <c r="R54" s="4"/>
+    </row>
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B55" s="3"/>
+      <c r="C55" s="3"/>
+      <c r="D55" s="3"/>
+      <c r="E55" s="3"/>
+      <c r="F55" s="3"/>
+      <c r="G55" s="3"/>
+      <c r="H55" s="3"/>
+      <c r="I55" s="3"/>
+      <c r="J55" s="4"/>
+      <c r="K55" s="4"/>
+      <c r="L55" s="4"/>
+      <c r="M55" s="4"/>
+      <c r="N55" s="4"/>
+      <c r="O55" s="4"/>
+      <c r="P55" s="4"/>
+      <c r="Q55" s="4"/>
+      <c r="R55" s="4"/>
+    </row>
+    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B56" s="3"/>
+      <c r="C56" s="3"/>
+      <c r="D56" s="3"/>
+      <c r="E56" s="3"/>
+      <c r="F56" s="3"/>
+      <c r="G56" s="3"/>
+      <c r="H56" s="3"/>
+      <c r="I56" s="3"/>
+      <c r="J56" s="4"/>
+      <c r="K56" s="4"/>
+      <c r="L56" s="4"/>
+      <c r="M56" s="4"/>
+      <c r="N56" s="4"/>
+      <c r="O56" s="4"/>
+      <c r="P56" s="4"/>
+      <c r="Q56" s="4"/>
+      <c r="R56" s="4"/>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="3"/>
+      <c r="B57" s="3"/>
+      <c r="C57" s="3"/>
+      <c r="D57" s="3"/>
+      <c r="E57" s="3"/>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="H57" s="3"/>
+      <c r="I57" s="3"/>
+      <c r="J57" s="4"/>
+      <c r="K57" s="4"/>
+      <c r="L57" s="4"/>
+      <c r="M57" s="4"/>
+      <c r="N57" s="4"/>
+      <c r="O57" s="4"/>
+      <c r="P57" s="4"/>
+      <c r="Q57" s="4"/>
+      <c r="R57" s="4"/>
+    </row>
   </sheetData>
-  <mergeCells count="112">
+  <mergeCells count="154">
     <mergeCell ref="A6:R6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C7:I7"/>
@@ -1456,6 +1976,48 @@
     <mergeCell ref="A43:B43"/>
     <mergeCell ref="C43:I43"/>
     <mergeCell ref="K43:R43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="C44:I44"/>
+    <mergeCell ref="K44:R44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="C45:I45"/>
+    <mergeCell ref="K45:R45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="C46:I46"/>
+    <mergeCell ref="K46:R46"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="C47:I47"/>
+    <mergeCell ref="K47:R47"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="C48:I48"/>
+    <mergeCell ref="K48:R48"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="C49:I49"/>
+    <mergeCell ref="K49:R49"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="C50:I50"/>
+    <mergeCell ref="K50:R50"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="C51:I51"/>
+    <mergeCell ref="K51:R51"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="C52:I52"/>
+    <mergeCell ref="K52:R52"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="C53:I53"/>
+    <mergeCell ref="K53:R53"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="C54:I54"/>
+    <mergeCell ref="K54:R54"/>
+    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="C55:I55"/>
+    <mergeCell ref="K55:R55"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="C56:I56"/>
+    <mergeCell ref="K56:R56"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="C57:I57"/>
+    <mergeCell ref="K57:R57"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Added new content from stream the other day.
</commit_message>
<xml_diff>
--- a/_Projects/P1012202501-ESP32_Stepper_Controller/ProjectDocuments/test-logs/P1012202501-01 Test Plan Log.xlsx
+++ b/_Projects/P1012202501-ESP32_Stepper_Controller/ProjectDocuments/test-logs/P1012202501-01 Test Plan Log.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="148">
   <si>
     <t xml:space="preserve">Functional Requirements Checklist</t>
   </si>
@@ -410,6 +410,60 @@
   </si>
   <si>
     <t xml:space="preserve">Does the basic HelloWorld firmware program and function properly?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SST 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the UARTFTDI firmware and interface operate properly?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SST 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the red status LED flash at the proper rate?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SST 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the RS-485 interface function properly?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SST 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the input for CN3 terminal 1 operate properly?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SST 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the input for CN3 terminal 2 operate properly?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SST 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the input for CN3 terminal 3 operate properly?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SST 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the input for CN4 terminal 1 operate properly?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SST 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the input for CN4 terminal 2 operate properly?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SST 11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the input for CN4 terminal 3 operate properly?</t>
   </si>
 </sst>
 </file>
@@ -419,7 +473,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -440,6 +494,11 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -497,12 +556,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -520,6 +579,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -705,7 +768,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A7:R105"/>
+  <dimension ref="A7:R114"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2793,9 +2856,13 @@
       <c r="R103" s="4"/>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A104" s="3"/>
+      <c r="A104" s="3" t="s">
+        <v>130</v>
+      </c>
       <c r="B104" s="3"/>
-      <c r="C104" s="3"/>
+      <c r="C104" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D104" s="3"/>
       <c r="E104" s="3"/>
       <c r="F104" s="3"/>
@@ -2813,9 +2880,13 @@
       <c r="R104" s="4"/>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A105" s="3"/>
+      <c r="A105" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="B105" s="3"/>
-      <c r="C105" s="3"/>
+      <c r="C105" s="3" t="s">
+        <v>133</v>
+      </c>
       <c r="D105" s="3"/>
       <c r="E105" s="3"/>
       <c r="F105" s="3"/>
@@ -2832,8 +2903,216 @@
       <c r="Q105" s="4"/>
       <c r="R105" s="4"/>
     </row>
+    <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A106" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106" s="3"/>
+      <c r="C106" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106" s="3"/>
+      <c r="E106" s="3"/>
+      <c r="F106" s="3"/>
+      <c r="G106" s="3"/>
+      <c r="H106" s="3"/>
+      <c r="I106" s="3"/>
+      <c r="J106" s="4"/>
+      <c r="K106" s="4"/>
+      <c r="L106" s="4"/>
+      <c r="M106" s="4"/>
+      <c r="N106" s="4"/>
+      <c r="O106" s="4"/>
+      <c r="P106" s="4"/>
+      <c r="Q106" s="4"/>
+      <c r="R106" s="4"/>
+    </row>
+    <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A107" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107" s="3"/>
+      <c r="C107" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="D107" s="3"/>
+      <c r="E107" s="3"/>
+      <c r="F107" s="3"/>
+      <c r="G107" s="3"/>
+      <c r="H107" s="3"/>
+      <c r="I107" s="3"/>
+      <c r="J107" s="4"/>
+      <c r="K107" s="4"/>
+      <c r="L107" s="4"/>
+      <c r="M107" s="4"/>
+      <c r="N107" s="4"/>
+      <c r="O107" s="4"/>
+      <c r="P107" s="4"/>
+      <c r="Q107" s="4"/>
+      <c r="R107" s="4"/>
+    </row>
+    <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A108" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B108" s="3"/>
+      <c r="C108" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D108" s="3"/>
+      <c r="E108" s="3"/>
+      <c r="F108" s="3"/>
+      <c r="G108" s="3"/>
+      <c r="H108" s="3"/>
+      <c r="I108" s="3"/>
+      <c r="J108" s="4"/>
+      <c r="K108" s="4"/>
+      <c r="L108" s="4"/>
+      <c r="M108" s="4"/>
+      <c r="N108" s="4"/>
+      <c r="O108" s="4"/>
+      <c r="P108" s="4"/>
+      <c r="Q108" s="4"/>
+      <c r="R108" s="4"/>
+    </row>
+    <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A109" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B109" s="3"/>
+      <c r="C109" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D109" s="6"/>
+      <c r="E109" s="6"/>
+      <c r="F109" s="6"/>
+      <c r="G109" s="6"/>
+      <c r="H109" s="6"/>
+      <c r="I109" s="6"/>
+      <c r="J109" s="4"/>
+      <c r="K109" s="4"/>
+      <c r="L109" s="4"/>
+      <c r="M109" s="4"/>
+      <c r="N109" s="4"/>
+      <c r="O109" s="4"/>
+      <c r="P109" s="4"/>
+      <c r="Q109" s="4"/>
+      <c r="R109" s="4"/>
+    </row>
+    <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A110" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B110" s="3"/>
+      <c r="C110" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="D110" s="6"/>
+      <c r="E110" s="6"/>
+      <c r="F110" s="6"/>
+      <c r="G110" s="6"/>
+      <c r="H110" s="6"/>
+      <c r="I110" s="6"/>
+      <c r="J110" s="4"/>
+      <c r="K110" s="4"/>
+      <c r="L110" s="4"/>
+      <c r="M110" s="4"/>
+      <c r="N110" s="4"/>
+      <c r="O110" s="4"/>
+      <c r="P110" s="4"/>
+      <c r="Q110" s="4"/>
+      <c r="R110" s="4"/>
+    </row>
+    <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A111" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B111" s="3"/>
+      <c r="C111" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="D111" s="6"/>
+      <c r="E111" s="6"/>
+      <c r="F111" s="6"/>
+      <c r="G111" s="6"/>
+      <c r="H111" s="6"/>
+      <c r="I111" s="6"/>
+      <c r="J111" s="4"/>
+      <c r="K111" s="4"/>
+      <c r="L111" s="4"/>
+      <c r="M111" s="4"/>
+      <c r="N111" s="4"/>
+      <c r="O111" s="4"/>
+      <c r="P111" s="4"/>
+      <c r="Q111" s="4"/>
+      <c r="R111" s="4"/>
+    </row>
+    <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A112" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="B112" s="3"/>
+      <c r="C112" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="D112" s="6"/>
+      <c r="E112" s="6"/>
+      <c r="F112" s="6"/>
+      <c r="G112" s="6"/>
+      <c r="H112" s="6"/>
+      <c r="I112" s="6"/>
+      <c r="J112" s="4"/>
+      <c r="K112" s="4"/>
+      <c r="L112" s="4"/>
+      <c r="M112" s="4"/>
+      <c r="N112" s="4"/>
+      <c r="O112" s="4"/>
+      <c r="P112" s="4"/>
+      <c r="Q112" s="4"/>
+      <c r="R112" s="4"/>
+    </row>
+    <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A113" s="3"/>
+      <c r="B113" s="3"/>
+      <c r="C113" s="3"/>
+      <c r="D113" s="3"/>
+      <c r="E113" s="3"/>
+      <c r="F113" s="3"/>
+      <c r="G113" s="3"/>
+      <c r="H113" s="3"/>
+      <c r="I113" s="3"/>
+      <c r="J113" s="4"/>
+      <c r="K113" s="4"/>
+      <c r="L113" s="4"/>
+      <c r="M113" s="4"/>
+      <c r="N113" s="4"/>
+      <c r="O113" s="4"/>
+      <c r="P113" s="4"/>
+      <c r="Q113" s="4"/>
+      <c r="R113" s="4"/>
+    </row>
+    <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A114" s="3"/>
+      <c r="B114" s="3"/>
+      <c r="C114" s="3"/>
+      <c r="D114" s="3"/>
+      <c r="E114" s="3"/>
+      <c r="F114" s="3"/>
+      <c r="G114" s="3"/>
+      <c r="H114" s="3"/>
+      <c r="I114" s="3"/>
+      <c r="J114" s="4"/>
+      <c r="K114" s="4"/>
+      <c r="L114" s="4"/>
+      <c r="M114" s="4"/>
+      <c r="N114" s="4"/>
+      <c r="O114" s="4"/>
+      <c r="P114" s="4"/>
+      <c r="Q114" s="4"/>
+      <c r="R114" s="4"/>
+    </row>
   </sheetData>
-  <mergeCells count="268">
+  <mergeCells count="295">
     <mergeCell ref="A7:R7"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="C8:I8"/>
@@ -3102,6 +3381,33 @@
     <mergeCell ref="A105:B105"/>
     <mergeCell ref="C105:I105"/>
     <mergeCell ref="K105:R105"/>
+    <mergeCell ref="A106:B106"/>
+    <mergeCell ref="C106:I106"/>
+    <mergeCell ref="K106:R106"/>
+    <mergeCell ref="A107:B107"/>
+    <mergeCell ref="C107:I107"/>
+    <mergeCell ref="K107:R107"/>
+    <mergeCell ref="A108:B108"/>
+    <mergeCell ref="C108:I108"/>
+    <mergeCell ref="K108:R108"/>
+    <mergeCell ref="A109:B109"/>
+    <mergeCell ref="C109:I109"/>
+    <mergeCell ref="K109:R109"/>
+    <mergeCell ref="A110:B110"/>
+    <mergeCell ref="C110:I110"/>
+    <mergeCell ref="K110:R110"/>
+    <mergeCell ref="A111:B111"/>
+    <mergeCell ref="C111:I111"/>
+    <mergeCell ref="K111:R111"/>
+    <mergeCell ref="A112:B112"/>
+    <mergeCell ref="C112:I112"/>
+    <mergeCell ref="K112:R112"/>
+    <mergeCell ref="A113:B113"/>
+    <mergeCell ref="C113:I113"/>
+    <mergeCell ref="K113:R113"/>
+    <mergeCell ref="A114:B114"/>
+    <mergeCell ref="C114:I114"/>
+    <mergeCell ref="K114:R114"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Added recent files from stream.
</commit_message>
<xml_diff>
--- a/_Projects/P1012202501-ESP32_Stepper_Controller/ProjectDocuments/test-logs/P1012202501-01 Test Plan Log.xlsx
+++ b/_Projects/P1012202501-ESP32_Stepper_Controller/ProjectDocuments/test-logs/P1012202501-01 Test Plan Log.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="152">
   <si>
     <t xml:space="preserve">Functional Requirements Checklist</t>
   </si>
@@ -464,6 +464,18 @@
   </si>
   <si>
     <t xml:space="preserve">Does the input for CN4 terminal 3 operate properly?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SST 12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do the inputs operate properly using a PLC as a control source?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SST 13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the stepper motor driver IC operate properly?</t>
   </si>
 </sst>
 </file>
@@ -473,7 +485,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -494,11 +506,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -556,7 +563,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -579,10 +586,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2980,15 +2983,15 @@
         <v>140</v>
       </c>
       <c r="B109" s="3"/>
-      <c r="C109" s="6" t="s">
+      <c r="C109" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="D109" s="6"/>
-      <c r="E109" s="6"/>
-      <c r="F109" s="6"/>
-      <c r="G109" s="6"/>
-      <c r="H109" s="6"/>
-      <c r="I109" s="6"/>
+      <c r="D109" s="3"/>
+      <c r="E109" s="3"/>
+      <c r="F109" s="3"/>
+      <c r="G109" s="3"/>
+      <c r="H109" s="3"/>
+      <c r="I109" s="3"/>
       <c r="J109" s="4"/>
       <c r="K109" s="4"/>
       <c r="L109" s="4"/>
@@ -3004,15 +3007,15 @@
         <v>142</v>
       </c>
       <c r="B110" s="3"/>
-      <c r="C110" s="6" t="s">
+      <c r="C110" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="D110" s="6"/>
-      <c r="E110" s="6"/>
-      <c r="F110" s="6"/>
-      <c r="G110" s="6"/>
-      <c r="H110" s="6"/>
-      <c r="I110" s="6"/>
+      <c r="D110" s="3"/>
+      <c r="E110" s="3"/>
+      <c r="F110" s="3"/>
+      <c r="G110" s="3"/>
+      <c r="H110" s="3"/>
+      <c r="I110" s="3"/>
       <c r="J110" s="4"/>
       <c r="K110" s="4"/>
       <c r="L110" s="4"/>
@@ -3028,15 +3031,15 @@
         <v>144</v>
       </c>
       <c r="B111" s="3"/>
-      <c r="C111" s="6" t="s">
+      <c r="C111" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="D111" s="6"/>
-      <c r="E111" s="6"/>
-      <c r="F111" s="6"/>
-      <c r="G111" s="6"/>
-      <c r="H111" s="6"/>
-      <c r="I111" s="6"/>
+      <c r="D111" s="3"/>
+      <c r="E111" s="3"/>
+      <c r="F111" s="3"/>
+      <c r="G111" s="3"/>
+      <c r="H111" s="3"/>
+      <c r="I111" s="3"/>
       <c r="J111" s="4"/>
       <c r="K111" s="4"/>
       <c r="L111" s="4"/>
@@ -3052,15 +3055,15 @@
         <v>146</v>
       </c>
       <c r="B112" s="3"/>
-      <c r="C112" s="6" t="s">
+      <c r="C112" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="D112" s="6"/>
-      <c r="E112" s="6"/>
-      <c r="F112" s="6"/>
-      <c r="G112" s="6"/>
-      <c r="H112" s="6"/>
-      <c r="I112" s="6"/>
+      <c r="D112" s="3"/>
+      <c r="E112" s="3"/>
+      <c r="F112" s="3"/>
+      <c r="G112" s="3"/>
+      <c r="H112" s="3"/>
+      <c r="I112" s="3"/>
       <c r="J112" s="4"/>
       <c r="K112" s="4"/>
       <c r="L112" s="4"/>
@@ -3072,9 +3075,13 @@
       <c r="R112" s="4"/>
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A113" s="3"/>
+      <c r="A113" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="B113" s="3"/>
-      <c r="C113" s="3"/>
+      <c r="C113" s="3" t="s">
+        <v>149</v>
+      </c>
       <c r="D113" s="3"/>
       <c r="E113" s="3"/>
       <c r="F113" s="3"/>
@@ -3092,9 +3099,13 @@
       <c r="R113" s="4"/>
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A114" s="3"/>
+      <c r="A114" s="3" t="s">
+        <v>150</v>
+      </c>
       <c r="B114" s="3"/>
-      <c r="C114" s="3"/>
+      <c r="C114" s="3" t="s">
+        <v>151</v>
+      </c>
       <c r="D114" s="3"/>
       <c r="E114" s="3"/>
       <c r="F114" s="3"/>

</xml_diff>